<commit_message>
added link groups file
</commit_message>
<xml_diff>
--- a/sample_data/Tutor_Copy_-_Fall_2026_Acceptance___Placement_Choices_for_LRC.xlsx
+++ b/sample_data/Tutor_Copy_-_Fall_2026_Acceptance___Placement_Choices_for_LRC.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Andre\tutor_assignment_app\sample_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\tutor_assignment_app\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3D88E67-A052-43F0-8D53-71EA7465115D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A6DE31-6C68-43E3-991F-4B30EC5E290A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Placements (Tutors Please Revie" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2541" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2605" uniqueCount="465">
   <si>
     <t>Tutors: Please review your placement(s) and Accept no later than Sunday Aug 16
 If for some reason your availability has changed, you must email LRC Pro Staff ASAP
@@ -1441,6 +1441,66 @@
   </si>
   <si>
     <t>Kassidy Saffa, Jasmine Torres, Ryan Moses (Tuesday only)</t>
+  </si>
+  <si>
+    <t>Link Group</t>
+  </si>
+  <si>
+    <t>BIOL 201 - A</t>
+  </si>
+  <si>
+    <t>BIOL 302 - A</t>
+  </si>
+  <si>
+    <t>COMP 121 - A</t>
+  </si>
+  <si>
+    <t>COMP 151 - A</t>
+  </si>
+  <si>
+    <t>COMP 162 - A</t>
+  </si>
+  <si>
+    <t>COMP 232 - A</t>
+  </si>
+  <si>
+    <t>COMP 262 - A</t>
+  </si>
+  <si>
+    <t>ESRM 203 - A</t>
+  </si>
+  <si>
+    <t>PSY 300 - A</t>
+  </si>
+  <si>
+    <t>PSY 301 - A</t>
+  </si>
+  <si>
+    <t>PSY 314 - A</t>
+  </si>
+  <si>
+    <t>PSY 300 - B</t>
+  </si>
+  <si>
+    <t>PSY 300 - C</t>
+  </si>
+  <si>
+    <t>PSY 300 - D</t>
+  </si>
+  <si>
+    <t>PSY 301 - B</t>
+  </si>
+  <si>
+    <t>PSY 314 - B</t>
+  </si>
+  <si>
+    <t>PSY 301 - C</t>
+  </si>
+  <si>
+    <t>PSY 314 - C</t>
+  </si>
+  <si>
+    <t>PSY 314 - D</t>
   </si>
 </sst>
 </file>
@@ -6551,7 +6611,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N157"/>
+  <dimension ref="A1:O157"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="16.90625" customWidth="1"/>
@@ -6566,6 +6626,7 @@
     <col min="10" max="10" width="20.36328125" customWidth="1"/>
     <col min="11" max="11" width="18.6328125" customWidth="1"/>
     <col min="13" max="13" width="17.90625" customWidth="1"/>
+    <col min="15" max="15" width="17.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="12.5">
@@ -6918,7 +6979,7 @@
       <c r="M16" s="120"/>
       <c r="N16" s="120"/>
     </row>
-    <row r="17" spans="1:14" ht="12.5">
+    <row r="17" spans="1:15" ht="12.5">
       <c r="A17" s="48"/>
       <c r="B17" s="146"/>
       <c r="C17" s="120"/>
@@ -6934,7 +6995,7 @@
       <c r="M17" s="48"/>
       <c r="N17" s="48"/>
     </row>
-    <row r="18" spans="1:14" ht="15.5">
+    <row r="18" spans="1:15" ht="16" thickBot="1">
       <c r="A18" s="52"/>
       <c r="B18" s="16" t="s">
         <v>39</v>
@@ -6975,8 +7036,11 @@
       <c r="N18" s="18" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" ht="15.5">
+      <c r="O18" s="18" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="16" thickTop="1">
       <c r="A19" s="24" t="s">
         <v>55</v>
       </c>
@@ -7016,7 +7080,7 @@
         <v>2502</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15.5">
+    <row r="20" spans="1:15" ht="15.5">
       <c r="A20" s="24" t="s">
         <v>55</v>
       </c>
@@ -7054,7 +7118,7 @@
         <v>1908</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.5">
+    <row r="21" spans="1:15" ht="15.5">
       <c r="A21" s="24" t="s">
         <v>55</v>
       </c>
@@ -7092,7 +7156,7 @@
         <v>1908</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15.5">
+    <row r="22" spans="1:15" ht="15.5">
       <c r="A22" s="24" t="s">
         <v>55</v>
       </c>
@@ -7130,7 +7194,7 @@
         <v>2330</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.5">
+    <row r="23" spans="1:15" ht="15.5">
       <c r="A23" s="24" t="s">
         <v>55</v>
       </c>
@@ -7170,7 +7234,7 @@
         <v>2582</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15.5">
+    <row r="24" spans="1:15" ht="15.5">
       <c r="A24" s="24" t="s">
         <v>74</v>
       </c>
@@ -7208,7 +7272,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15.5">
+    <row r="25" spans="1:15" ht="15.5">
       <c r="A25" s="24" t="s">
         <v>74</v>
       </c>
@@ -7246,7 +7310,7 @@
         <v>1360</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="15.5">
+    <row r="26" spans="1:15" ht="15.5">
       <c r="A26" s="24" t="s">
         <v>55</v>
       </c>
@@ -7283,8 +7347,11 @@
       <c r="N26" s="63">
         <v>1411</v>
       </c>
-    </row>
-    <row r="27" spans="1:14" ht="15.5">
+      <c r="O26" s="63" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="15.5">
       <c r="A27" s="24" t="s">
         <v>55</v>
       </c>
@@ -7321,8 +7388,11 @@
       <c r="N27" s="63">
         <v>134</v>
       </c>
-    </row>
-    <row r="28" spans="1:14" ht="15.5">
+      <c r="O27" s="63" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="15.5">
       <c r="A28" s="24" t="s">
         <v>55</v>
       </c>
@@ -7359,8 +7429,11 @@
       <c r="N28" s="63">
         <v>134</v>
       </c>
-    </row>
-    <row r="29" spans="1:14" ht="15.5">
+      <c r="O28" s="63" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="15.5">
       <c r="A29" s="24" t="s">
         <v>57</v>
       </c>
@@ -7402,7 +7475,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="31">
+    <row r="30" spans="1:15" ht="31">
       <c r="A30" s="24" t="s">
         <v>57</v>
       </c>
@@ -7442,7 +7515,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15.5">
+    <row r="31" spans="1:15" ht="15.5">
       <c r="A31" s="24" t="s">
         <v>74</v>
       </c>
@@ -7480,7 +7553,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="62">
+    <row r="32" spans="1:15" ht="62">
       <c r="A32" s="24" t="s">
         <v>74</v>
       </c>
@@ -7524,7 +7597,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="46.5">
+    <row r="33" spans="1:15" ht="46.5">
       <c r="A33" s="24" t="s">
         <v>74</v>
       </c>
@@ -7566,7 +7639,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="15.5">
+    <row r="34" spans="1:15" ht="15.5">
       <c r="A34" s="24" t="s">
         <v>55</v>
       </c>
@@ -7604,7 +7677,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="15.5">
+    <row r="35" spans="1:15" ht="15.5">
       <c r="A35" s="24" t="s">
         <v>74</v>
       </c>
@@ -7642,7 +7715,7 @@
         <v>1535</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="15.5">
+    <row r="36" spans="1:15" ht="15.5">
       <c r="A36" s="24" t="s">
         <v>74</v>
       </c>
@@ -7680,7 +7753,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="31">
+    <row r="37" spans="1:15" ht="31">
       <c r="A37" s="24" t="s">
         <v>74</v>
       </c>
@@ -7721,8 +7794,11 @@
       <c r="N37" s="63">
         <v>1422</v>
       </c>
-    </row>
-    <row r="38" spans="1:14" ht="15.5">
+      <c r="O37" s="63" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15" ht="15.5">
       <c r="A38" s="24" t="s">
         <v>74</v>
       </c>
@@ -7761,8 +7837,11 @@
       <c r="N38" s="63">
         <v>1422</v>
       </c>
-    </row>
-    <row r="39" spans="1:14" ht="15.5">
+      <c r="O38" s="63" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15" ht="15.5">
       <c r="A39" s="24" t="s">
         <v>74</v>
       </c>
@@ -7798,7 +7877,7 @@
       </c>
       <c r="N39" s="63"/>
     </row>
-    <row r="40" spans="1:14" ht="15.5">
+    <row r="40" spans="1:15" ht="15.5">
       <c r="A40" s="24" t="s">
         <v>74</v>
       </c>
@@ -7834,7 +7913,7 @@
       </c>
       <c r="N40" s="63"/>
     </row>
-    <row r="41" spans="1:14" ht="15.5">
+    <row r="41" spans="1:15" ht="15.5">
       <c r="A41" s="24" t="s">
         <v>74</v>
       </c>
@@ -7872,7 +7951,7 @@
         <v>2582</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="15.5">
+    <row r="42" spans="1:15" ht="15.5">
       <c r="A42" s="24" t="s">
         <v>74</v>
       </c>
@@ -7914,7 +7993,7 @@
         <v>1642</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="15.5">
+    <row r="43" spans="1:15" ht="15.5">
       <c r="A43" s="24" t="s">
         <v>74</v>
       </c>
@@ -7954,7 +8033,7 @@
         <v>3540</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="15.5">
+    <row r="44" spans="1:15" ht="15.5">
       <c r="A44" s="24" t="s">
         <v>74</v>
       </c>
@@ -7992,7 +8071,7 @@
         <v>2572</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="31">
+    <row r="45" spans="1:15" ht="31">
       <c r="A45" s="24" t="s">
         <v>74</v>
       </c>
@@ -8036,7 +8115,7 @@
         <v>1411</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="31">
+    <row r="46" spans="1:15" ht="31">
       <c r="A46" s="24" t="s">
         <v>74</v>
       </c>
@@ -8078,7 +8157,7 @@
         <v>1462</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="15.5">
+    <row r="47" spans="1:15" ht="15.5">
       <c r="A47" s="24" t="s">
         <v>74</v>
       </c>
@@ -8122,7 +8201,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="31">
+    <row r="48" spans="1:15" ht="31">
       <c r="A48" s="24" t="s">
         <v>74</v>
       </c>
@@ -8162,7 +8241,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="15.5">
+    <row r="49" spans="1:15" ht="15.5">
       <c r="A49" s="24" t="s">
         <v>74</v>
       </c>
@@ -8200,7 +8279,7 @@
         <v>2570</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="31">
+    <row r="50" spans="1:15" ht="31">
       <c r="A50" s="24" t="s">
         <v>74</v>
       </c>
@@ -8244,7 +8323,7 @@
         <v>1545</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="46.5">
+    <row r="51" spans="1:15" ht="46.5">
       <c r="A51" s="24" t="s">
         <v>74</v>
       </c>
@@ -8286,7 +8365,7 @@
         <v>2572</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="15.5">
+    <row r="52" spans="1:15" ht="15.5">
       <c r="A52" s="24" t="s">
         <v>57</v>
       </c>
@@ -8330,7 +8409,7 @@
         <v>3570</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="15.5">
+    <row r="53" spans="1:15" ht="15.5">
       <c r="A53" s="24" t="s">
         <v>55</v>
       </c>
@@ -8369,8 +8448,11 @@
       <c r="N53" s="63">
         <v>1501</v>
       </c>
-    </row>
-    <row r="54" spans="1:14" ht="15.5">
+      <c r="O53" s="63" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="54" spans="1:15" ht="15.5">
       <c r="A54" s="24" t="s">
         <v>55</v>
       </c>
@@ -8409,8 +8491,11 @@
       <c r="N54" s="63">
         <v>3570</v>
       </c>
-    </row>
-    <row r="55" spans="1:14" ht="15.5">
+      <c r="O54" s="63" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" ht="15.5">
       <c r="A55" s="24" t="s">
         <v>55</v>
       </c>
@@ -8449,8 +8534,11 @@
       <c r="N55" s="63">
         <v>3570</v>
       </c>
-    </row>
-    <row r="56" spans="1:14" ht="15.5">
+      <c r="O55" s="63" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="56" spans="1:15" ht="15.5">
       <c r="A56" s="24" t="s">
         <v>57</v>
       </c>
@@ -8494,7 +8582,7 @@
         <v>3570</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15.5">
+    <row r="57" spans="1:15" ht="15.5">
       <c r="A57" s="24" t="s">
         <v>74</v>
       </c>
@@ -8531,8 +8619,11 @@
         <v>178</v>
       </c>
       <c r="N57" s="63"/>
-    </row>
-    <row r="58" spans="1:14" ht="15.5">
+      <c r="O57" s="63" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="58" spans="1:15" ht="15.5">
       <c r="A58" s="78" t="s">
         <v>74</v>
       </c>
@@ -8570,7 +8661,7 @@
       </c>
       <c r="N58" s="81"/>
     </row>
-    <row r="59" spans="1:14" ht="15.5">
+    <row r="59" spans="1:15" ht="15.5">
       <c r="A59" s="24" t="s">
         <v>74</v>
       </c>
@@ -8609,8 +8700,11 @@
         <v>178</v>
       </c>
       <c r="N59" s="63"/>
-    </row>
-    <row r="60" spans="1:14" ht="15.5">
+      <c r="O59" s="63" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="60" spans="1:15" ht="15.5">
       <c r="A60" s="24" t="s">
         <v>74</v>
       </c>
@@ -8649,8 +8743,11 @@
       <c r="N60" s="63">
         <v>1411</v>
       </c>
-    </row>
-    <row r="61" spans="1:14" ht="31">
+      <c r="O60" s="63" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="61" spans="1:15" ht="31">
       <c r="A61" s="24" t="s">
         <v>74</v>
       </c>
@@ -8691,8 +8788,11 @@
       <c r="N61" s="63">
         <v>3540</v>
       </c>
-    </row>
-    <row r="62" spans="1:14" ht="15.5">
+      <c r="O61" s="63" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" ht="15.5">
       <c r="A62" s="24" t="s">
         <v>74</v>
       </c>
@@ -8729,8 +8829,11 @@
       <c r="N62" s="63">
         <v>3540</v>
       </c>
-    </row>
-    <row r="63" spans="1:14" ht="15.5">
+      <c r="O62" s="63" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" ht="15.5">
       <c r="A63" s="24" t="s">
         <v>74</v>
       </c>
@@ -8771,8 +8874,11 @@
       <c r="N63" s="63">
         <v>1462</v>
       </c>
-    </row>
-    <row r="64" spans="1:14" ht="15.5">
+      <c r="O63" s="63" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" ht="15.5">
       <c r="A64" s="24" t="s">
         <v>74</v>
       </c>
@@ -8813,8 +8919,11 @@
       <c r="N64" s="63">
         <v>1232</v>
       </c>
-    </row>
-    <row r="65" spans="1:14" ht="15.5">
+      <c r="O64" s="63" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="65" spans="1:15" ht="15.5">
       <c r="A65" s="24" t="s">
         <v>74</v>
       </c>
@@ -8853,8 +8962,11 @@
       <c r="N65" s="63">
         <v>1232</v>
       </c>
-    </row>
-    <row r="66" spans="1:14" ht="15.5">
+      <c r="O65" s="63" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" ht="15.5">
       <c r="A66" s="24" t="s">
         <v>55</v>
       </c>
@@ -8895,8 +9007,11 @@
       <c r="N66" s="63">
         <v>2550</v>
       </c>
-    </row>
-    <row r="67" spans="1:14" ht="15.5">
+      <c r="O66" s="63" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" ht="15.5">
       <c r="A67" s="24" t="s">
         <v>55</v>
       </c>
@@ -8935,8 +9050,11 @@
       <c r="N67" s="63">
         <v>3540</v>
       </c>
-    </row>
-    <row r="68" spans="1:14" ht="15.5">
+      <c r="O67" s="63" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" ht="15.5">
       <c r="A68" s="84" t="s">
         <v>55</v>
       </c>
@@ -8978,7 +9096,7 @@
         <v>3540</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="15.5">
+    <row r="69" spans="1:15" ht="15.5">
       <c r="A69" s="24" t="s">
         <v>57</v>
       </c>
@@ -9022,7 +9140,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="15.5">
+    <row r="70" spans="1:15" ht="15.5">
       <c r="A70" s="24" t="s">
         <v>57</v>
       </c>
@@ -9064,7 +9182,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="15.5">
+    <row r="71" spans="1:15" ht="15.5">
       <c r="A71" s="24" t="s">
         <v>74</v>
       </c>
@@ -9106,7 +9224,7 @@
         <v>2582</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="15.5">
+    <row r="72" spans="1:15" ht="15.5">
       <c r="A72" s="24" t="s">
         <v>74</v>
       </c>
@@ -9146,7 +9264,7 @@
         <v>2530</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="15.5">
+    <row r="73" spans="1:15" ht="15.5">
       <c r="A73" s="24" t="s">
         <v>74</v>
       </c>
@@ -9184,7 +9302,7 @@
         <v>2330</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="31">
+    <row r="74" spans="1:15" ht="31">
       <c r="A74" s="24" t="s">
         <v>57</v>
       </c>
@@ -9223,8 +9341,11 @@
       <c r="N74" s="63">
         <v>2432</v>
       </c>
-    </row>
-    <row r="75" spans="1:14" ht="15.5">
+      <c r="O74" s="63" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" ht="15.5">
       <c r="A75" s="24" t="s">
         <v>57</v>
       </c>
@@ -9261,8 +9382,11 @@
       <c r="N75" s="63">
         <v>2432</v>
       </c>
-    </row>
-    <row r="76" spans="1:14" ht="15.5">
+      <c r="O75" s="63" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" ht="15.5">
       <c r="A76" s="24" t="s">
         <v>57</v>
       </c>
@@ -9304,7 +9428,7 @@
         <v>3550</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="31">
+    <row r="77" spans="1:15" ht="31">
       <c r="A77" s="24" t="s">
         <v>57</v>
       </c>
@@ -9348,7 +9472,7 @@
         <v>3501</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="31">
+    <row r="78" spans="1:15" ht="31">
       <c r="A78" s="24" t="s">
         <v>57</v>
       </c>
@@ -9388,7 +9512,7 @@
         <v>1550</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="31">
+    <row r="79" spans="1:15" ht="31">
       <c r="A79" s="24" t="s">
         <v>57</v>
       </c>
@@ -9430,7 +9554,7 @@
         <v>2598</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="31">
+    <row r="80" spans="1:15" ht="31">
       <c r="A80" s="24" t="s">
         <v>57</v>
       </c>
@@ -10810,7 +10934,7 @@
         <v>2411</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="15.5">
+    <row r="113" spans="1:15" ht="15.5">
       <c r="A113" s="24" t="s">
         <v>74</v>
       </c>
@@ -10852,7 +10976,7 @@
         <v>2411</v>
       </c>
     </row>
-    <row r="114" spans="1:14" ht="15.5">
+    <row r="114" spans="1:15" ht="15.5">
       <c r="A114" s="24" t="s">
         <v>55</v>
       </c>
@@ -10889,8 +11013,11 @@
       <c r="N114" s="63">
         <v>1411</v>
       </c>
-    </row>
-    <row r="115" spans="1:14" ht="15.5">
+      <c r="O114" s="63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="115" spans="1:15" ht="15.5">
       <c r="A115" s="24" t="s">
         <v>55</v>
       </c>
@@ -10927,8 +11054,11 @@
       <c r="N115" s="63">
         <v>1360</v>
       </c>
-    </row>
-    <row r="116" spans="1:14" ht="15.5">
+      <c r="O115" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="116" spans="1:15" ht="15.5">
       <c r="A116" s="24" t="s">
         <v>92</v>
       </c>
@@ -10963,8 +11093,11 @@
         <v>178</v>
       </c>
       <c r="N116" s="63"/>
-    </row>
-    <row r="117" spans="1:14" ht="15.5">
+      <c r="O116" s="63" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="117" spans="1:15" ht="15.5">
       <c r="A117" s="24" t="s">
         <v>92</v>
       </c>
@@ -10997,8 +11130,11 @@
         <v>178</v>
       </c>
       <c r="N117" s="63"/>
-    </row>
-    <row r="118" spans="1:14" ht="15.5">
+      <c r="O117" s="63" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="118" spans="1:15" ht="15.5">
       <c r="A118" s="24" t="s">
         <v>55</v>
       </c>
@@ -11035,8 +11171,11 @@
       <c r="N118" s="63">
         <v>3314</v>
       </c>
-    </row>
-    <row r="119" spans="1:14" ht="15.5">
+      <c r="O118" s="63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="119" spans="1:15" ht="15.5">
       <c r="A119" s="24" t="s">
         <v>55</v>
       </c>
@@ -11073,8 +11212,11 @@
       <c r="N119" s="63">
         <v>3314</v>
       </c>
-    </row>
-    <row r="120" spans="1:14" ht="15.5">
+      <c r="O119" s="63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="120" spans="1:15" ht="15.5">
       <c r="A120" s="24" t="s">
         <v>55</v>
       </c>
@@ -11111,8 +11253,11 @@
       <c r="N120" s="63">
         <v>3314</v>
       </c>
-    </row>
-    <row r="121" spans="1:14" ht="15.5">
+      <c r="O120" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="121" spans="1:15" ht="15.5">
       <c r="A121" s="24" t="s">
         <v>55</v>
       </c>
@@ -11149,8 +11294,11 @@
       <c r="N121" s="63">
         <v>3314</v>
       </c>
-    </row>
-    <row r="122" spans="1:14" ht="15.5">
+      <c r="O121" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="122" spans="1:15" ht="15.5">
       <c r="A122" s="24" t="s">
         <v>55</v>
       </c>
@@ -11185,8 +11333,11 @@
         <v>178</v>
       </c>
       <c r="N122" s="63"/>
-    </row>
-    <row r="123" spans="1:14" ht="15.5">
+      <c r="O122" s="63" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="123" spans="1:15" ht="15.5">
       <c r="A123" s="24" t="s">
         <v>55</v>
       </c>
@@ -11221,8 +11372,11 @@
         <v>178</v>
       </c>
       <c r="N123" s="63"/>
-    </row>
-    <row r="124" spans="1:14" ht="15.5">
+      <c r="O123" s="63" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="124" spans="1:15" ht="15.5">
       <c r="A124" s="24" t="s">
         <v>55</v>
       </c>
@@ -11257,8 +11411,11 @@
         <v>178</v>
       </c>
       <c r="N124" s="63"/>
-    </row>
-    <row r="125" spans="1:14" ht="15.5">
+      <c r="O124" s="63" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="125" spans="1:15" ht="15.5">
       <c r="A125" s="24" t="s">
         <v>55</v>
       </c>
@@ -11293,8 +11450,11 @@
         <v>178</v>
       </c>
       <c r="N125" s="63"/>
-    </row>
-    <row r="126" spans="1:14" ht="15.5">
+      <c r="O125" s="63" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="126" spans="1:15" ht="15.5">
       <c r="A126" s="24" t="s">
         <v>92</v>
       </c>
@@ -11331,8 +11491,11 @@
       <c r="N126" s="63">
         <v>2515</v>
       </c>
-    </row>
-    <row r="127" spans="1:14" ht="15.5">
+      <c r="O126" s="63" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="127" spans="1:15" ht="15.5">
       <c r="A127" s="24" t="s">
         <v>92</v>
       </c>
@@ -11365,8 +11528,11 @@
         <v>178</v>
       </c>
       <c r="N127" s="63"/>
-    </row>
-    <row r="128" spans="1:14" ht="15.5">
+      <c r="O127" s="63" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="128" spans="1:15" ht="15.5">
       <c r="A128" s="24" t="s">
         <v>92</v>
       </c>
@@ -11399,8 +11565,11 @@
         <v>178</v>
       </c>
       <c r="N128" s="63"/>
-    </row>
-    <row r="129" spans="1:14" ht="15.5">
+      <c r="O128" s="63" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="129" spans="1:15" ht="15.5">
       <c r="A129" s="24" t="s">
         <v>55</v>
       </c>
@@ -11437,8 +11606,11 @@
       <c r="N129" s="63">
         <v>3344</v>
       </c>
-    </row>
-    <row r="130" spans="1:14" ht="15.5">
+      <c r="O129" s="63" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="130" spans="1:15" ht="15.5">
       <c r="A130" s="24" t="s">
         <v>55</v>
       </c>
@@ -11475,8 +11647,11 @@
       <c r="N130" s="63">
         <v>3344</v>
       </c>
-    </row>
-    <row r="131" spans="1:14" ht="15.5">
+      <c r="O130" s="63" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="131" spans="1:15" ht="15.5">
       <c r="A131" s="24" t="s">
         <v>55</v>
       </c>
@@ -11513,8 +11688,11 @@
       <c r="N131" s="63">
         <v>3314</v>
       </c>
-    </row>
-    <row r="132" spans="1:14" ht="15.5">
+      <c r="O131" s="63" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="132" spans="1:15" ht="15.5">
       <c r="A132" s="24" t="s">
         <v>55</v>
       </c>
@@ -11549,8 +11727,11 @@
         <v>178</v>
       </c>
       <c r="N132" s="63"/>
-    </row>
-    <row r="133" spans="1:14" ht="15.5">
+      <c r="O132" s="63" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="133" spans="1:15" ht="15.5">
       <c r="A133" s="24" t="s">
         <v>55</v>
       </c>
@@ -11585,8 +11766,11 @@
         <v>178</v>
       </c>
       <c r="N133" s="63"/>
-    </row>
-    <row r="134" spans="1:14" ht="15.5">
+      <c r="O133" s="63" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="134" spans="1:15" ht="15.5">
       <c r="A134" s="24" t="s">
         <v>55</v>
       </c>
@@ -11625,8 +11809,11 @@
       <c r="N134" s="63">
         <v>1501</v>
       </c>
-    </row>
-    <row r="135" spans="1:14" ht="15.5">
+      <c r="O134" s="63" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="135" spans="1:15" ht="15.5">
       <c r="A135" s="24" t="s">
         <v>55</v>
       </c>
@@ -11665,8 +11852,11 @@
       <c r="N135" s="63">
         <v>3332</v>
       </c>
-    </row>
-    <row r="136" spans="1:14" ht="15.5">
+      <c r="O135" s="63" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="136" spans="1:15" ht="15.5">
       <c r="A136" s="24" t="s">
         <v>55</v>
       </c>
@@ -11699,8 +11889,11 @@
         <v>178</v>
       </c>
       <c r="N136" s="63"/>
-    </row>
-    <row r="137" spans="1:14" ht="15.5">
+      <c r="O136" s="63" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="137" spans="1:15" ht="15.5">
       <c r="A137" s="24" t="s">
         <v>55</v>
       </c>
@@ -11733,8 +11926,11 @@
         <v>178</v>
       </c>
       <c r="N137" s="63"/>
-    </row>
-    <row r="138" spans="1:14" ht="15.5">
+      <c r="O137" s="63" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="138" spans="1:15" ht="15.5">
       <c r="A138" s="24" t="s">
         <v>55</v>
       </c>
@@ -11773,8 +11969,11 @@
       <c r="N138" s="63">
         <v>3332</v>
       </c>
-    </row>
-    <row r="139" spans="1:14" ht="15.5">
+      <c r="O138" s="63" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="139" spans="1:15" ht="15.5">
       <c r="A139" s="24" t="s">
         <v>55</v>
       </c>
@@ -11811,8 +12010,11 @@
       <c r="N139" s="63">
         <v>3332</v>
       </c>
-    </row>
-    <row r="140" spans="1:14" ht="31">
+      <c r="O139" s="63" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="140" spans="1:15" ht="31">
       <c r="A140" s="24" t="s">
         <v>55</v>
       </c>
@@ -11851,8 +12053,11 @@
       <c r="N140" s="63">
         <v>3332</v>
       </c>
-    </row>
-    <row r="141" spans="1:14" ht="15.5">
+      <c r="O140" s="63" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="141" spans="1:15" ht="15.5">
       <c r="A141" s="24" t="s">
         <v>55</v>
       </c>
@@ -11885,8 +12090,11 @@
         <v>178</v>
       </c>
       <c r="N141" s="63"/>
-    </row>
-    <row r="142" spans="1:14" ht="15.5">
+      <c r="O141" s="63" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="142" spans="1:15" ht="15.5">
       <c r="A142" s="24" t="s">
         <v>55</v>
       </c>
@@ -11919,8 +12127,11 @@
         <v>178</v>
       </c>
       <c r="N142" s="63"/>
-    </row>
-    <row r="143" spans="1:14" ht="15.5">
+      <c r="O142" s="63" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="143" spans="1:15" ht="15.5">
       <c r="A143" s="24" t="s">
         <v>55</v>
       </c>
@@ -11953,8 +12164,11 @@
         <v>178</v>
       </c>
       <c r="N143" s="63"/>
-    </row>
-    <row r="144" spans="1:14" ht="15.5">
+      <c r="O143" s="63" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="144" spans="1:15" ht="15.5">
       <c r="A144" s="24" t="s">
         <v>55</v>
       </c>
@@ -11987,8 +12201,11 @@
         <v>178</v>
       </c>
       <c r="N144" s="63"/>
-    </row>
-    <row r="145" spans="1:14" ht="41.25" customHeight="1">
+      <c r="O144" s="63" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="145" spans="1:15" ht="41.25" customHeight="1">
       <c r="A145" s="24"/>
       <c r="B145" s="138" t="s">
         <v>431</v>
@@ -12006,7 +12223,7 @@
       <c r="M145" s="120"/>
       <c r="N145" s="120"/>
     </row>
-    <row r="146" spans="1:14" ht="15.5">
+    <row r="146" spans="1:15" ht="15.5">
       <c r="A146" s="24" t="s">
         <v>92</v>
       </c>
@@ -12041,8 +12258,11 @@
         <v>178</v>
       </c>
       <c r="N146" s="63"/>
-    </row>
-    <row r="147" spans="1:14" ht="15.5">
+      <c r="O146" s="63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="147" spans="1:15" ht="15.5">
       <c r="A147" s="24" t="s">
         <v>92</v>
       </c>
@@ -12079,8 +12299,11 @@
         <v>178</v>
       </c>
       <c r="N147" s="63"/>
-    </row>
-    <row r="148" spans="1:14" ht="15.5">
+      <c r="O147" s="63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="148" spans="1:15" ht="15.5">
       <c r="A148" s="24" t="s">
         <v>92</v>
       </c>
@@ -12113,8 +12336,11 @@
         <v>178</v>
       </c>
       <c r="N148" s="63"/>
-    </row>
-    <row r="149" spans="1:14" ht="15.5">
+      <c r="O148" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="149" spans="1:15" ht="15.5">
       <c r="A149" s="24" t="s">
         <v>406</v>
       </c>
@@ -12149,8 +12375,11 @@
         <v>178</v>
       </c>
       <c r="N149" s="63"/>
-    </row>
-    <row r="150" spans="1:14" ht="15.5">
+      <c r="O149" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="150" spans="1:15" ht="15.5">
       <c r="A150" s="24" t="s">
         <v>406</v>
       </c>
@@ -12189,8 +12418,11 @@
         <v>178</v>
       </c>
       <c r="N150" s="63"/>
-    </row>
-    <row r="151" spans="1:14" ht="15.5">
+      <c r="O150" s="63" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="151" spans="1:15" ht="15.5">
       <c r="A151" s="24" t="s">
         <v>92</v>
       </c>
@@ -12223,8 +12455,11 @@
         <v>178</v>
       </c>
       <c r="N151" s="63"/>
-    </row>
-    <row r="152" spans="1:14" ht="15.5">
+      <c r="O151" s="63" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="152" spans="1:15" ht="15.5">
       <c r="A152" s="24" t="s">
         <v>406</v>
       </c>
@@ -12261,8 +12496,11 @@
         <v>178</v>
       </c>
       <c r="N152" s="63"/>
-    </row>
-    <row r="153" spans="1:14" ht="15.5">
+      <c r="O152" s="63" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="153" spans="1:15" ht="15.5">
       <c r="A153" s="24" t="s">
         <v>92</v>
       </c>
@@ -12295,8 +12533,11 @@
         <v>178</v>
       </c>
       <c r="N153" s="63"/>
-    </row>
-    <row r="154" spans="1:14" ht="15.5">
+      <c r="O153" s="63" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="154" spans="1:15" ht="15.5">
       <c r="A154" s="24" t="s">
         <v>406</v>
       </c>
@@ -12333,8 +12574,11 @@
         <v>178</v>
       </c>
       <c r="N154" s="63"/>
-    </row>
-    <row r="155" spans="1:14" ht="15.5">
+      <c r="O154" s="63" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="155" spans="1:15" ht="15.5">
       <c r="A155" s="24" t="s">
         <v>92</v>
       </c>
@@ -12371,8 +12615,11 @@
         <v>178</v>
       </c>
       <c r="N155" s="63"/>
-    </row>
-    <row r="156" spans="1:14" ht="15.5">
+      <c r="O155" s="63" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="156" spans="1:15" ht="15.5">
       <c r="A156" s="24" t="s">
         <v>92</v>
       </c>
@@ -12409,8 +12656,11 @@
         <v>178</v>
       </c>
       <c r="N156" s="63"/>
-    </row>
-    <row r="157" spans="1:14" ht="15.5">
+      <c r="O156" s="63" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="157" spans="1:15" ht="15.5">
       <c r="A157" s="24" t="s">
         <v>92</v>
       </c>
@@ -12445,6 +12695,9 @@
         <v>178</v>
       </c>
       <c r="N157" s="63"/>
+      <c r="O157" s="63" t="s">
+        <v>456</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="16">

</xml_diff>